<commit_message>
time data to molecules
</commit_message>
<xml_diff>
--- a/experiments/results.xlsx
+++ b/experiments/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lvuorenk/Documents/vaikkari/paulioptnew/pauliopt/experiments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{707D1B80-5C91-E24D-8E35-DF7B4D479676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF60BB9-8A8F-1047-AB02-BDE973443D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17240" xr2:uid="{85E89CC3-FE57-2C44-8224-50BF94C0E0C4}"/>
+    <workbookView xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17240" activeTab="2" xr2:uid="{85E89CC3-FE57-2C44-8224-50BF94C0E0C4}"/>
   </bookViews>
   <sheets>
     <sheet name="line6" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="72">
   <si>
     <t>gadgets</t>
   </si>
@@ -249,6 +249,15 @@
   <si>
     <t>pauli strings</t>
   </si>
+  <si>
+    <t>time do</t>
+  </si>
+  <si>
+    <t>time diff</t>
+  </si>
+  <si>
+    <t>time lo</t>
+  </si>
 </sst>
 </file>
 
@@ -257,7 +266,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -394,6 +403,12 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -751,7 +766,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -760,6 +775,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -13632,16 +13652,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>368300</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>330200</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>107950</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -17661,1237 +17681,1603 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F53CADA0-3FD9-B748-A167-0AF6A36FD04E}">
-  <dimension ref="C3:L44"/>
+  <dimension ref="B1:M45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="5" max="5" width="7.1640625" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="5.83203125" customWidth="1"/>
+    <col min="5" max="5" width="9.1640625" customWidth="1"/>
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="0" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="10" width="0" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1640625" customWidth="1"/>
+    <col min="8" max="8" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.83203125" customWidth="1"/>
     <col min="11" max="11" width="7.83203125" customWidth="1"/>
     <col min="12" max="12" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="I1" s="8"/>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B3" s="4" t="s">
+        <v>60</v>
+      </c>
       <c r="C3" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="4" t="s">
         <v>15</v>
       </c>
+      <c r="D3" s="5" t="s">
+        <v>61</v>
+      </c>
       <c r="E3" s="5" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>64</v>
       </c>
       <c r="I3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="5"/>
       <c r="K3" s="5" t="s">
         <v>65</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="4" spans="3:12" x14ac:dyDescent="0.2">
+      <c r="M3" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
       <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
         <v>19</v>
       </c>
+      <c r="D4">
+        <v>14</v>
+      </c>
       <c r="E4">
-        <v>14</v>
+        <v>1488</v>
       </c>
       <c r="F4">
-        <v>1488</v>
+        <v>7641</v>
       </c>
       <c r="G4">
-        <v>7955</v>
+        <v>115.21801499999999</v>
       </c>
       <c r="H4">
         <v>12419</v>
       </c>
       <c r="I4">
-        <v>10850</v>
+        <v>273.029291</v>
+      </c>
+      <c r="J4">
+        <v>10625</v>
       </c>
       <c r="K4" s="3">
-        <f t="shared" ref="K4:K19" si="0">G4/H4-1</f>
-        <v>-0.35944923101699011</v>
+        <f>F4/H4-1</f>
+        <v>-0.38473307029551496</v>
       </c>
       <c r="L4" s="1">
-        <f t="shared" ref="L4:L19" si="1">I4/G4-1</f>
-        <v>0.36392206159648022</v>
-      </c>
-    </row>
-    <row r="5" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J4/F4-1</f>
+        <v>0.39052480041879334</v>
+      </c>
+      <c r="M4" s="3">
+        <f>G4/I4-1</f>
+        <v>-0.57800126653810202</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
       <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s">
         <v>19</v>
       </c>
+      <c r="D5">
+        <v>14</v>
+      </c>
       <c r="E5">
-        <v>14</v>
+        <v>1488</v>
       </c>
       <c r="F5">
-        <v>1488</v>
+        <v>5000</v>
       </c>
       <c r="G5">
-        <v>5059</v>
+        <v>81.148252999999997</v>
       </c>
       <c r="H5">
         <v>12181</v>
       </c>
       <c r="I5">
-        <v>8081</v>
+        <v>284.52725500000003</v>
+      </c>
+      <c r="J5">
+        <v>8085</v>
       </c>
       <c r="K5" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.58468106066825376</v>
+        <f>F5/H5-1</f>
+        <v>-0.58952466956735905</v>
       </c>
       <c r="L5" s="1">
-        <f t="shared" si="1"/>
-        <v>0.59735125518877252</v>
-      </c>
-    </row>
-    <row r="6" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J5/F5-1</f>
+        <v>0.61699999999999999</v>
+      </c>
+      <c r="M5" s="3">
+        <f>G5/I5-1</f>
+        <v>-0.71479620467290561</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
       <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
         <v>19</v>
       </c>
+      <c r="D6">
+        <v>12</v>
+      </c>
       <c r="E6">
-        <v>12</v>
+        <v>1085</v>
       </c>
       <c r="F6">
-        <v>1085</v>
+        <v>3133</v>
       </c>
       <c r="G6">
-        <v>3672</v>
+        <v>33.076317000000003</v>
       </c>
       <c r="H6">
         <v>8482</v>
       </c>
       <c r="I6">
-        <v>3058</v>
+        <v>129.12428800000001</v>
+      </c>
+      <c r="J6">
+        <v>3160</v>
       </c>
       <c r="K6" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.56708323508606462</v>
-      </c>
-      <c r="L6" s="3">
-        <f t="shared" si="1"/>
-        <v>-0.16721132897603486</v>
-      </c>
-    </row>
-    <row r="7" spans="3:12" x14ac:dyDescent="0.2">
+        <f>F6/H6-1</f>
+        <v>-0.63062956849799567</v>
+      </c>
+      <c r="L6" s="1">
+        <f>J6/F6-1</f>
+        <v>8.6179380785189608E-3</v>
+      </c>
+      <c r="M6" s="3">
+        <f>G6/I6-1</f>
+        <v>-0.74384124387195072</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
       <c r="C7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" t="s">
         <v>22</v>
       </c>
+      <c r="D7">
+        <v>18</v>
+      </c>
       <c r="E7">
-        <v>18</v>
+        <v>2950</v>
       </c>
       <c r="F7">
-        <v>2950</v>
+        <v>21046</v>
       </c>
       <c r="G7">
-        <v>22858</v>
+        <v>461.34287899999998</v>
       </c>
       <c r="H7">
         <v>37786</v>
       </c>
       <c r="I7">
-        <v>15037</v>
+        <v>2522.6866450000002</v>
+      </c>
+      <c r="J7">
+        <v>14622</v>
       </c>
       <c r="K7" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.39506695601545549</v>
+        <f>F7/H7-1</f>
+        <v>-0.44302122479225114</v>
       </c>
       <c r="L7" s="3">
-        <f t="shared" si="1"/>
-        <v>-0.34215591915303178</v>
-      </c>
-    </row>
-    <row r="8" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J7/F7-1</f>
+        <v>-0.3052361493870569</v>
+      </c>
+      <c r="M7" s="3">
+        <f>G7/I7-1</f>
+        <v>-0.81712240007517867</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
       <c r="C8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" t="s">
         <v>19</v>
       </c>
+      <c r="D8">
+        <v>14</v>
+      </c>
       <c r="E8">
-        <v>14</v>
+        <v>1488</v>
       </c>
       <c r="F8">
-        <v>1488</v>
+        <v>7893</v>
       </c>
       <c r="G8">
-        <v>6958</v>
+        <v>132.73884000000001</v>
       </c>
       <c r="H8">
         <v>12919</v>
       </c>
       <c r="I8">
-        <v>9138</v>
+        <v>346.42907000000002</v>
+      </c>
+      <c r="J8">
+        <v>8778</v>
       </c>
       <c r="K8" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.46141342209149316</v>
+        <f>F8/H8-1</f>
+        <v>-0.38903939933431375</v>
       </c>
       <c r="L8" s="1">
-        <f t="shared" si="1"/>
-        <v>0.31330842196033348</v>
-      </c>
-    </row>
-    <row r="9" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J8/F8-1</f>
+        <v>0.11212466742683391</v>
+      </c>
+      <c r="M8" s="3">
+        <f>G8/I8-1</f>
+        <v>-0.61683688958319816</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
       <c r="C9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" t="s">
         <v>19</v>
       </c>
+      <c r="D9">
+        <v>14</v>
+      </c>
       <c r="E9">
-        <v>14</v>
+        <v>1488</v>
       </c>
       <c r="F9">
-        <v>1488</v>
+        <v>10567</v>
       </c>
       <c r="G9">
-        <v>10715</v>
+        <v>161.85106200000001</v>
       </c>
       <c r="H9">
         <v>13433</v>
       </c>
       <c r="I9">
-        <v>6682</v>
+        <v>306.45082100000002</v>
+      </c>
+      <c r="J9">
+        <v>7464</v>
       </c>
       <c r="K9" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.20233752698578134</v>
+        <f>F9/H9-1</f>
+        <v>-0.21335517010347649</v>
       </c>
       <c r="L9" s="3">
-        <f t="shared" si="1"/>
-        <v>-0.37638824078394773</v>
-      </c>
-    </row>
-    <row r="10" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J9/F9-1</f>
+        <v>-0.29365004258540739</v>
+      </c>
+      <c r="M9" s="3">
+        <f>G9/I9-1</f>
+        <v>-0.47185306447588204</v>
+      </c>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
       <c r="C10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" t="s">
         <v>19</v>
       </c>
+      <c r="D10">
+        <v>12</v>
+      </c>
       <c r="E10">
-        <v>12</v>
+        <v>2109</v>
       </c>
       <c r="F10">
-        <v>2109</v>
+        <v>4962</v>
       </c>
       <c r="G10">
-        <v>4975</v>
+        <v>85.607489999999999</v>
       </c>
       <c r="H10">
         <v>14909</v>
       </c>
       <c r="I10">
-        <v>4839</v>
+        <v>560.85743500000001</v>
+      </c>
+      <c r="J10">
+        <v>4532</v>
       </c>
       <c r="K10" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.66630894090817627</v>
+        <f>F10/H10-1</f>
+        <v>-0.6671808974444966</v>
       </c>
       <c r="L10" s="3">
-        <f t="shared" si="1"/>
-        <v>-2.7336683417085395E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J10/F10-1</f>
+        <v>-8.6658605401047972E-2</v>
+      </c>
+      <c r="M10" s="3">
+        <f>G10/I10-1</f>
+        <v>-0.84736318954209811</v>
+      </c>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
       <c r="C11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" t="s">
         <v>19</v>
       </c>
+      <c r="D11">
+        <v>14</v>
+      </c>
       <c r="E11">
-        <v>14</v>
+        <v>1000</v>
       </c>
       <c r="F11">
-        <v>1000</v>
+        <v>5320</v>
       </c>
       <c r="G11">
-        <v>4527</v>
+        <v>49.378607000000002</v>
       </c>
       <c r="H11">
         <v>8675</v>
       </c>
       <c r="I11">
-        <v>7127</v>
+        <v>105.78508100000001</v>
+      </c>
+      <c r="J11">
+        <v>7590</v>
       </c>
       <c r="K11" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.47815561959654174</v>
+        <f>F11/H11-1</f>
+        <v>-0.3867435158501441</v>
       </c>
       <c r="L11" s="1">
-        <f t="shared" si="1"/>
-        <v>0.57433178705544519</v>
-      </c>
-    </row>
-    <row r="12" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J11/F11-1</f>
+        <v>0.42669172932330834</v>
+      </c>
+      <c r="M11" s="3">
+        <f>G11/I11-1</f>
+        <v>-0.53321766610926924</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
       <c r="C12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" t="s">
         <v>19</v>
       </c>
+      <c r="D12">
+        <v>14</v>
+      </c>
       <c r="E12">
-        <v>14</v>
+        <v>1000</v>
       </c>
       <c r="F12">
-        <v>1000</v>
+        <v>4252</v>
       </c>
       <c r="G12">
-        <v>4983</v>
+        <v>36.524329999999999</v>
       </c>
       <c r="H12">
         <v>7967</v>
       </c>
       <c r="I12">
-        <v>3450</v>
+        <v>87.638071999999994</v>
+      </c>
+      <c r="J12">
+        <v>3406</v>
       </c>
       <c r="K12" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.37454499811723363</v>
+        <f>F12/H12-1</f>
+        <v>-0.46629848123509476</v>
       </c>
       <c r="L12" s="3">
-        <f t="shared" si="1"/>
-        <v>-0.30764599638771828</v>
-      </c>
-    </row>
-    <row r="13" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J12/F12-1</f>
+        <v>-0.19896519285042336</v>
+      </c>
+      <c r="M12" s="3">
+        <f>G12/I12-1</f>
+        <v>-0.58323672387498438</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
       <c r="C13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" t="s">
         <v>19</v>
       </c>
+      <c r="D13">
+        <v>12</v>
+      </c>
       <c r="E13">
-        <v>12</v>
+        <v>1085</v>
       </c>
       <c r="F13">
-        <v>1085</v>
+        <v>3222</v>
       </c>
       <c r="G13">
-        <v>3129</v>
+        <v>23.810727</v>
       </c>
       <c r="H13">
         <v>8077</v>
       </c>
       <c r="I13">
-        <v>2872</v>
+        <v>90.031066999999993</v>
+      </c>
+      <c r="J13">
+        <v>2767</v>
       </c>
       <c r="K13" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.6126036894886715</v>
+        <f>F13/H13-1</f>
+        <v>-0.60108951343320538</v>
       </c>
       <c r="L13" s="3">
-        <f t="shared" si="1"/>
-        <v>-8.2134867369766718E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J13/F13-1</f>
+        <v>-0.1412166356300435</v>
+      </c>
+      <c r="M13" s="3">
+        <f>G13/I13-1</f>
+        <v>-0.73552765957999799</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>30</v>
+      </c>
       <c r="C14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" t="s">
         <v>19</v>
       </c>
+      <c r="D14">
+        <v>8</v>
+      </c>
       <c r="E14">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="F14">
-        <v>84</v>
+        <v>289</v>
       </c>
       <c r="G14">
-        <v>298</v>
+        <v>0.19081300000000001</v>
       </c>
       <c r="H14">
         <v>443</v>
       </c>
       <c r="I14">
-        <v>271</v>
+        <v>0.279721</v>
+      </c>
+      <c r="J14">
+        <v>266</v>
       </c>
       <c r="K14" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.32731376975169302</v>
+        <f>F14/H14-1</f>
+        <v>-0.34762979683972917</v>
       </c>
       <c r="L14" s="3">
-        <f t="shared" si="1"/>
-        <v>-9.060402684563762E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J14/F14-1</f>
+        <v>-7.9584775086505188E-2</v>
+      </c>
+      <c r="M14" s="3">
+        <f>G14/I14-1</f>
+        <v>-0.31784528154839997</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
       <c r="C15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" t="s">
         <v>32</v>
       </c>
+      <c r="D15">
+        <v>4</v>
+      </c>
       <c r="E15">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F15">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="G15">
-        <v>22</v>
+        <v>1.486E-2</v>
       </c>
       <c r="H15">
         <v>35</v>
       </c>
       <c r="I15">
+        <v>5.5510000000000004E-3</v>
+      </c>
+      <c r="J15">
         <v>24</v>
       </c>
       <c r="K15" s="3">
-        <f t="shared" si="0"/>
+        <f>F15/H15-1</f>
         <v>-0.37142857142857144</v>
       </c>
       <c r="L15" s="1">
-        <f t="shared" si="1"/>
+        <f>J15/F15-1</f>
         <v>9.0909090909090828E-2</v>
       </c>
-    </row>
-    <row r="16" spans="3:12" x14ac:dyDescent="0.2">
+      <c r="M15" s="7">
+        <f>G15/I15-1</f>
+        <v>1.6769951360115294</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
       <c r="C16" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" t="s">
         <v>19</v>
       </c>
+      <c r="D16">
+        <v>8</v>
+      </c>
       <c r="E16">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="F16">
-        <v>84</v>
+        <v>327</v>
       </c>
       <c r="G16">
-        <v>317</v>
+        <v>0.27967599999999998</v>
       </c>
       <c r="H16">
         <v>414</v>
       </c>
       <c r="I16">
-        <v>267</v>
+        <v>0.30827500000000002</v>
+      </c>
+      <c r="J16">
+        <v>247</v>
       </c>
       <c r="K16" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.2342995169082126</v>
+        <f>F16/H16-1</f>
+        <v>-0.21014492753623193</v>
       </c>
       <c r="L16" s="3">
-        <f t="shared" si="1"/>
-        <v>-0.1577287066246057</v>
-      </c>
-    </row>
-    <row r="17" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J16/F16-1</f>
+        <v>-0.24464831804281351</v>
+      </c>
+      <c r="M16" s="3">
+        <f>G16/I16-1</f>
+        <v>-9.2771064796042579E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
       <c r="C17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" t="s">
         <v>32</v>
       </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
       <c r="E17">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F17">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G17">
-        <v>24</v>
+        <v>1.1167E-2</v>
       </c>
       <c r="H17">
         <v>38</v>
       </c>
       <c r="I17">
+        <v>6.3090000000000004E-3</v>
+      </c>
+      <c r="J17">
         <v>29</v>
       </c>
       <c r="K17" s="3">
-        <f t="shared" si="0"/>
+        <f>F17/H17-1</f>
         <v>-0.36842105263157898</v>
       </c>
       <c r="L17" s="1">
-        <f t="shared" si="1"/>
+        <f>J17/F17-1</f>
         <v>0.20833333333333326</v>
       </c>
-    </row>
-    <row r="18" spans="3:12" x14ac:dyDescent="0.2">
+      <c r="M17" s="7">
+        <f>G17/I17-1</f>
+        <v>0.77001109526073841</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
       <c r="C18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D18" t="s">
         <v>36</v>
       </c>
+      <c r="D18">
+        <v>6</v>
+      </c>
       <c r="E18">
-        <v>6</v>
+        <v>158</v>
       </c>
       <c r="F18">
-        <v>158</v>
+        <v>237</v>
       </c>
       <c r="G18">
-        <v>235</v>
+        <v>0.26958500000000002</v>
       </c>
       <c r="H18">
         <v>433</v>
       </c>
       <c r="I18">
+        <v>0.34162100000000001</v>
+      </c>
+      <c r="J18">
         <v>215</v>
       </c>
       <c r="K18" s="3">
-        <f t="shared" si="0"/>
-        <v>-0.45727482678983833</v>
+        <f>F18/H18-1</f>
+        <v>-0.45265588914549648</v>
       </c>
       <c r="L18" s="3">
-        <f t="shared" si="1"/>
-        <v>-8.5106382978723416E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="3:12" x14ac:dyDescent="0.2">
+        <f>J18/F18-1</f>
+        <v>-9.2827004219409259E-2</v>
+      </c>
+      <c r="M18" s="3">
+        <f>G18/I18-1</f>
+        <v>-0.210865257112414</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
       <c r="C19" t="s">
-        <v>37</v>
-      </c>
-      <c r="D19" t="s">
         <v>32</v>
       </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
       <c r="E19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G19">
-        <v>5</v>
+        <v>5.1599999999999997E-3</v>
       </c>
       <c r="H19">
         <v>5</v>
       </c>
       <c r="I19">
+        <v>2.0890000000000001E-3</v>
+      </c>
+      <c r="J19">
         <v>2</v>
       </c>
-      <c r="K19" s="1">
-        <f t="shared" si="0"/>
+      <c r="K19" s="7">
+        <f>F19/H19-1</f>
         <v>0</v>
       </c>
       <c r="L19" s="3">
-        <f t="shared" si="1"/>
+        <f>J19/F19-1</f>
         <v>-0.6</v>
       </c>
-    </row>
-    <row r="20" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="K20" s="1"/>
-      <c r="L20" s="3"/>
-    </row>
-    <row r="21" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C21" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="G21" s="5" t="s">
+      <c r="M19" s="7">
+        <f>G19/I19-1</f>
+        <v>1.4700813786500713</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20">
         <v>16</v>
       </c>
-      <c r="H21" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="L21" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="22" spans="3:12" x14ac:dyDescent="0.2">
+      <c r="E20">
+        <v>1440</v>
+      </c>
+      <c r="F20">
+        <v>11382</v>
+      </c>
+      <c r="G20">
+        <v>164.80469600000001</v>
+      </c>
+      <c r="H20">
+        <v>13852</v>
+      </c>
+      <c r="I20">
+        <v>378.60474699999997</v>
+      </c>
+      <c r="J20">
+        <v>11815</v>
+      </c>
+      <c r="K20" s="3">
+        <f>F20/H20-1</f>
+        <v>-0.17831360092405424</v>
+      </c>
+      <c r="L20" s="1">
+        <f>J20/F20-1</f>
+        <v>3.8042523282375784E-2</v>
+      </c>
+      <c r="M20" s="3">
+        <f>G20/I20-1</f>
+        <v>-0.56470515146499201</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21">
+        <v>8</v>
+      </c>
+      <c r="E21">
+        <v>160</v>
+      </c>
+      <c r="F21">
+        <v>448</v>
+      </c>
+      <c r="G21">
+        <v>0.668852</v>
+      </c>
+      <c r="H21">
+        <v>878</v>
+      </c>
+      <c r="I21">
+        <v>1.1275869999999999</v>
+      </c>
+      <c r="J21">
+        <v>382</v>
+      </c>
+      <c r="K21" s="3">
+        <f>F21/H21-1</f>
+        <v>-0.48974943052391795</v>
+      </c>
+      <c r="L21" s="3">
+        <f>J21/F21-1</f>
+        <v>-0.1473214285714286</v>
+      </c>
+      <c r="M21" s="3">
+        <f>G21/I21-1</f>
+        <v>-0.40682891874418559</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>40</v>
+      </c>
       <c r="C22" t="s">
-        <v>38</v>
-      </c>
-      <c r="D22" t="s">
         <v>22</v>
       </c>
+      <c r="D22">
+        <v>16</v>
+      </c>
       <c r="E22">
+        <v>1440</v>
+      </c>
+      <c r="F22">
+        <v>11626</v>
+      </c>
+      <c r="G22">
+        <v>165.386697</v>
+      </c>
+      <c r="H22">
+        <v>11727</v>
+      </c>
+      <c r="I22">
+        <v>309.21366599999999</v>
+      </c>
+      <c r="J22">
+        <v>6468</v>
+      </c>
+      <c r="K22" s="3">
+        <f>F22/H22-1</f>
+        <v>-8.6126033938773716E-3</v>
+      </c>
+      <c r="L22" s="3">
+        <f>J22/F22-1</f>
+        <v>-0.44366076036469981</v>
+      </c>
+      <c r="M22" s="3">
+        <f>G22/I22-1</f>
+        <v>-0.46513781509255803</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>41</v>
+      </c>
+      <c r="C23" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23">
+        <v>8</v>
+      </c>
+      <c r="E23">
+        <v>160</v>
+      </c>
+      <c r="F23">
+        <v>507</v>
+      </c>
+      <c r="G23">
+        <v>0.79593100000000006</v>
+      </c>
+      <c r="H23">
+        <v>883</v>
+      </c>
+      <c r="I23">
+        <v>1.149607</v>
+      </c>
+      <c r="J23">
+        <v>421</v>
+      </c>
+      <c r="K23" s="3">
+        <f>F23/H23-1</f>
+        <v>-0.42582106455266133</v>
+      </c>
+      <c r="L23" s="3">
+        <f>J23/F23-1</f>
+        <v>-0.16962524654832345</v>
+      </c>
+      <c r="M23" s="3">
+        <f>G23/I23-1</f>
+        <v>-0.30764948369312295</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24">
+        <v>14</v>
+      </c>
+      <c r="E24">
+        <v>2912</v>
+      </c>
+      <c r="F24">
+        <v>15866</v>
+      </c>
+      <c r="G24">
+        <v>318.762201</v>
+      </c>
+      <c r="H24">
+        <v>24224</v>
+      </c>
+      <c r="I24">
+        <v>1493.9029410000001</v>
+      </c>
+      <c r="J24">
+        <v>8374</v>
+      </c>
+      <c r="K24" s="3">
+        <f>F24/H24-1</f>
+        <v>-0.34502972258916775</v>
+      </c>
+      <c r="L24" s="3">
+        <f>J24/F24-1</f>
+        <v>-0.47220471448380186</v>
+      </c>
+      <c r="M24" s="3">
+        <f>G24/I24-1</f>
+        <v>-0.78662455755885685</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25">
+        <v>6</v>
+      </c>
+      <c r="E25">
+        <v>164</v>
+      </c>
+      <c r="F25">
+        <v>217</v>
+      </c>
+      <c r="G25">
+        <v>0.58277299999999999</v>
+      </c>
+      <c r="H25">
+        <v>471</v>
+      </c>
+      <c r="I25">
+        <v>0.57758100000000001</v>
+      </c>
+      <c r="J25">
+        <v>191</v>
+      </c>
+      <c r="K25" s="3">
+        <f>F25/H25-1</f>
+        <v>-0.53927813163481952</v>
+      </c>
+      <c r="L25" s="3">
+        <f>J25/F25-1</f>
+        <v>-0.11981566820276501</v>
+      </c>
+      <c r="M25" s="7">
+        <f>G25/I25-1</f>
+        <v>8.9892153654638207E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" t="s">
+        <v>22</v>
+      </c>
+      <c r="D26">
         <v>16</v>
       </c>
-      <c r="F22">
-        <v>1440</v>
-      </c>
-      <c r="G22">
-        <v>11580</v>
-      </c>
-      <c r="H22">
-        <v>13852</v>
-      </c>
-      <c r="I22">
-        <v>11196</v>
-      </c>
-      <c r="K22" s="3">
-        <f t="shared" ref="K22:K42" si="2">G22/H22-1</f>
-        <v>-0.16401963615362403</v>
-      </c>
-      <c r="L22" s="3">
-        <f t="shared" ref="L22:L42" si="3">I22/G22-1</f>
-        <v>-3.3160621761658016E-2</v>
-      </c>
-    </row>
-    <row r="23" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C23" t="s">
-        <v>39</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="E26">
+        <v>2688</v>
+      </c>
+      <c r="F26">
+        <v>20605</v>
+      </c>
+      <c r="G26">
+        <v>626.60672199999999</v>
+      </c>
+      <c r="H26">
+        <v>28018</v>
+      </c>
+      <c r="I26">
+        <v>1932.4593809999999</v>
+      </c>
+      <c r="J26">
+        <v>11809</v>
+      </c>
+      <c r="K26" s="3">
+        <f>F26/H26-1</f>
+        <v>-0.26457991291312732</v>
+      </c>
+      <c r="L26" s="3">
+        <f>J26/F26-1</f>
+        <v>-0.42688667799077895</v>
+      </c>
+      <c r="M26" s="3">
+        <f>G26/I26-1</f>
+        <v>-0.67574649787684204</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" t="s">
+        <v>22</v>
+      </c>
+      <c r="D27">
+        <v>16</v>
+      </c>
+      <c r="E27">
+        <v>2688</v>
+      </c>
+      <c r="F27">
+        <v>9143</v>
+      </c>
+      <c r="G27">
+        <v>335.78666199999998</v>
+      </c>
+      <c r="H27">
+        <v>29280</v>
+      </c>
+      <c r="I27">
+        <v>2134.8060519999999</v>
+      </c>
+      <c r="J27">
+        <v>10652</v>
+      </c>
+      <c r="K27" s="3">
+        <f>F27/H27-1</f>
+        <v>-0.68773907103825138</v>
+      </c>
+      <c r="L27" s="1">
+        <f>J27/F27-1</f>
+        <v>0.1650442961828722</v>
+      </c>
+      <c r="M27" s="3">
+        <f>G27/I27-1</f>
+        <v>-0.84270858625053213</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
+        <v>46</v>
+      </c>
+      <c r="C28" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28">
+        <v>20</v>
+      </c>
+      <c r="E28">
+        <v>684</v>
+      </c>
+      <c r="F28">
+        <v>4953</v>
+      </c>
+      <c r="G28">
+        <v>34.247933000000003</v>
+      </c>
+      <c r="H28">
+        <v>6308</v>
+      </c>
+      <c r="I28">
+        <v>60.474814000000002</v>
+      </c>
+      <c r="J28">
+        <v>4740</v>
+      </c>
+      <c r="K28" s="3">
+        <f>F28/H28-1</f>
+        <v>-0.21480659480025366</v>
+      </c>
+      <c r="L28" s="3">
+        <f>J28/F28-1</f>
+        <v>-4.300423985463353E-2</v>
+      </c>
+      <c r="M28" s="3">
+        <f>G28/I28-1</f>
+        <v>-0.43368270632465278</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B29" t="s">
+        <v>47</v>
+      </c>
+      <c r="C29" t="s">
+        <v>22</v>
+      </c>
+      <c r="D29">
+        <v>20</v>
+      </c>
+      <c r="E29">
+        <v>684</v>
+      </c>
+      <c r="F29">
+        <v>4946</v>
+      </c>
+      <c r="G29">
+        <v>32.466031000000001</v>
+      </c>
+      <c r="H29">
+        <v>5807</v>
+      </c>
+      <c r="I29">
+        <v>55.383809999999997</v>
+      </c>
+      <c r="J29">
+        <v>5704</v>
+      </c>
+      <c r="K29" s="3">
+        <f>F29/H29-1</f>
+        <v>-0.14826933011882215</v>
+      </c>
+      <c r="L29" s="1">
+        <f>J29/F29-1</f>
+        <v>0.15325515568135861</v>
+      </c>
+      <c r="M29" s="3">
+        <f>G29/I29-1</f>
+        <v>-0.41379924927519429</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" t="s">
+        <v>22</v>
+      </c>
+      <c r="D30">
+        <v>22</v>
+      </c>
+      <c r="E30">
+        <v>3240</v>
+      </c>
+      <c r="F30">
+        <v>42385</v>
+      </c>
+      <c r="G30">
+        <v>1592.0266979999999</v>
+      </c>
+      <c r="H30">
+        <v>35792</v>
+      </c>
+      <c r="I30">
+        <v>3037.7464949999999</v>
+      </c>
+      <c r="J30">
+        <v>47282</v>
+      </c>
+      <c r="K30" s="7">
+        <f>F30/H30-1</f>
+        <v>0.18420317389360741</v>
+      </c>
+      <c r="L30" s="1">
+        <f>J30/F30-1</f>
+        <v>0.11553615665919548</v>
+      </c>
+      <c r="M30" s="3">
+        <f>G30/I30-1</f>
+        <v>-0.47591851373364846</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" t="s">
         <v>19</v>
       </c>
-      <c r="E23">
-        <v>8</v>
-      </c>
-      <c r="F23">
-        <v>160</v>
-      </c>
-      <c r="G23">
-        <v>452</v>
-      </c>
-      <c r="H23">
-        <v>878</v>
-      </c>
-      <c r="I23">
-        <v>379</v>
-      </c>
-      <c r="K23" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.48519362186788151</v>
-      </c>
-      <c r="L23" s="3">
-        <f t="shared" si="3"/>
-        <v>-0.16150442477876104</v>
-      </c>
-    </row>
-    <row r="24" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C24" t="s">
-        <v>40</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="D31">
+        <v>12</v>
+      </c>
+      <c r="E31">
+        <v>640</v>
+      </c>
+      <c r="F31">
+        <v>2564</v>
+      </c>
+      <c r="G31">
+        <v>15.482094999999999</v>
+      </c>
+      <c r="H31">
+        <v>4250</v>
+      </c>
+      <c r="I31">
+        <v>28.972878999999999</v>
+      </c>
+      <c r="J31">
+        <v>3275</v>
+      </c>
+      <c r="K31" s="3">
+        <f>F31/H31-1</f>
+        <v>-0.39670588235294113</v>
+      </c>
+      <c r="L31" s="1">
+        <f>J31/F31-1</f>
+        <v>0.27730109204368181</v>
+      </c>
+      <c r="M31" s="3">
+        <f>G31/I31-1</f>
+        <v>-0.4656349132580162</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>50</v>
+      </c>
+      <c r="C32" t="s">
         <v>22</v>
       </c>
-      <c r="E24">
+      <c r="D32">
+        <v>22</v>
+      </c>
+      <c r="E32">
+        <v>3240</v>
+      </c>
+      <c r="F32">
+        <v>24416</v>
+      </c>
+      <c r="G32">
+        <v>852.84564499999999</v>
+      </c>
+      <c r="H32">
+        <v>33673</v>
+      </c>
+      <c r="I32">
+        <v>3113.253412</v>
+      </c>
+      <c r="J32">
+        <v>16037</v>
+      </c>
+      <c r="K32" s="3">
+        <f>F32/H32-1</f>
+        <v>-0.27490868054524398</v>
+      </c>
+      <c r="L32" s="3">
+        <f>J32/F32-1</f>
+        <v>-0.34317660550458717</v>
+      </c>
+      <c r="M32" s="3">
+        <f>G32/I32-1</f>
+        <v>-0.7260596770848412</v>
+      </c>
+    </row>
+    <row r="33" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>51</v>
+      </c>
+      <c r="C33" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33">
+        <v>12</v>
+      </c>
+      <c r="E33">
+        <v>640</v>
+      </c>
+      <c r="F33">
+        <v>2503</v>
+      </c>
+      <c r="G33">
+        <v>14.346698</v>
+      </c>
+      <c r="H33">
+        <v>4331</v>
+      </c>
+      <c r="I33">
+        <v>29.301047000000001</v>
+      </c>
+      <c r="J33">
+        <v>2336</v>
+      </c>
+      <c r="K33" s="3">
+        <f>F33/H33-1</f>
+        <v>-0.4220734241514662</v>
+      </c>
+      <c r="L33" s="3">
+        <f>J33/F33-1</f>
+        <v>-6.6719936076707897E-2</v>
+      </c>
+      <c r="M33" s="3">
+        <f>G33/I33-1</f>
+        <v>-0.51036910046251927</v>
+      </c>
+    </row>
+    <row r="34" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>52</v>
+      </c>
+      <c r="C34" t="s">
+        <v>19</v>
+      </c>
+      <c r="D34">
+        <v>10</v>
+      </c>
+      <c r="E34">
+        <v>630</v>
+      </c>
+      <c r="F34">
+        <v>1432</v>
+      </c>
+      <c r="G34">
+        <v>6.5066259999999998</v>
+      </c>
+      <c r="H34">
+        <v>3472</v>
+      </c>
+      <c r="I34">
+        <v>20.047049999999999</v>
+      </c>
+      <c r="J34">
+        <v>1468</v>
+      </c>
+      <c r="K34" s="3">
+        <f>F34/H34-1</f>
+        <v>-0.5875576036866359</v>
+      </c>
+      <c r="L34" s="1">
+        <f>J34/F34-1</f>
+        <v>2.5139664804469275E-2</v>
+      </c>
+      <c r="M34" s="3">
+        <f>G34/I34-1</f>
+        <v>-0.67543224564212689</v>
+      </c>
+    </row>
+    <row r="35" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B35" t="s">
+        <v>53</v>
+      </c>
+      <c r="C35" t="s">
+        <v>22</v>
+      </c>
+      <c r="D35">
+        <v>18</v>
+      </c>
+      <c r="E35">
+        <v>2950</v>
+      </c>
+      <c r="F35">
+        <v>21728</v>
+      </c>
+      <c r="G35">
+        <v>508.06735300000003</v>
+      </c>
+      <c r="H35">
+        <v>35602</v>
+      </c>
+      <c r="I35">
+        <v>2431.2650039999999</v>
+      </c>
+      <c r="J35">
+        <v>15910</v>
+      </c>
+      <c r="K35" s="3">
+        <f>F35/H35-1</f>
+        <v>-0.38969720802202124</v>
+      </c>
+      <c r="L35" s="3">
+        <f>J35/F35-1</f>
+        <v>-0.2677650957290133</v>
+      </c>
+      <c r="M35" s="3">
+        <f>G35/I35-1</f>
+        <v>-0.79102757117627642</v>
+      </c>
+    </row>
+    <row r="36" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
+        <v>54</v>
+      </c>
+      <c r="C36" t="s">
+        <v>22</v>
+      </c>
+      <c r="D36">
         <v>16</v>
       </c>
-      <c r="F24">
-        <v>1440</v>
-      </c>
-      <c r="G24">
-        <v>11701</v>
-      </c>
-      <c r="H24">
-        <v>11727</v>
-      </c>
-      <c r="I24">
-        <v>6813</v>
-      </c>
-      <c r="K24" s="1">
-        <f t="shared" si="2"/>
-        <v>-2.2171058241664543E-3</v>
-      </c>
-      <c r="L24" s="3">
-        <f t="shared" si="3"/>
-        <v>-0.41774207332706603</v>
-      </c>
-    </row>
-    <row r="25" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C25" t="s">
-        <v>41</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="E36">
+        <v>2340</v>
+      </c>
+      <c r="F36">
+        <v>19534</v>
+      </c>
+      <c r="G36">
+        <v>472.31464199999999</v>
+      </c>
+      <c r="H36">
+        <v>25280</v>
+      </c>
+      <c r="I36">
+        <v>1281.476625</v>
+      </c>
+      <c r="J36">
+        <v>13035</v>
+      </c>
+      <c r="K36" s="3">
+        <f>F36/H36-1</f>
+        <v>-0.2272943037974684</v>
+      </c>
+      <c r="L36" s="3">
+        <f>J36/F36-1</f>
+        <v>-0.33270195556465654</v>
+      </c>
+      <c r="M36" s="3">
+        <f>G36/I36-1</f>
+        <v>-0.63142937390683973</v>
+      </c>
+    </row>
+    <row r="37" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" t="s">
+        <v>22</v>
+      </c>
+      <c r="D37">
+        <v>16</v>
+      </c>
+      <c r="E37">
+        <v>2340</v>
+      </c>
+      <c r="F37">
+        <v>9597</v>
+      </c>
+      <c r="G37">
+        <v>222.20063200000001</v>
+      </c>
+      <c r="H37">
+        <v>23182</v>
+      </c>
+      <c r="I37">
+        <v>1149.347585</v>
+      </c>
+      <c r="J37">
+        <v>9670</v>
+      </c>
+      <c r="K37" s="3">
+        <f>F37/H37-1</f>
+        <v>-0.58601501164696745</v>
+      </c>
+      <c r="L37" s="1">
+        <f>J37/F37-1</f>
+        <v>7.6065437115764301E-3</v>
+      </c>
+      <c r="M37" s="3">
+        <f>G37/I37-1</f>
+        <v>-0.8066723810099623</v>
+      </c>
+    </row>
+    <row r="38" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>56</v>
+      </c>
+      <c r="C38" t="s">
         <v>19</v>
       </c>
-      <c r="E25">
-        <v>8</v>
-      </c>
-      <c r="F25">
-        <v>160</v>
-      </c>
-      <c r="G25">
-        <v>523</v>
-      </c>
-      <c r="H25">
-        <v>883</v>
-      </c>
-      <c r="I25">
-        <v>414</v>
-      </c>
-      <c r="K25" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.40770101925254809</v>
-      </c>
-      <c r="L25" s="3">
-        <f t="shared" si="3"/>
-        <v>-0.20841300191204593</v>
-      </c>
-    </row>
-    <row r="26" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C26" t="s">
-        <v>42</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="D38">
+        <v>12</v>
+      </c>
+      <c r="E38">
+        <v>640</v>
+      </c>
+      <c r="F38">
+        <v>2200</v>
+      </c>
+      <c r="G38">
+        <v>10.826136999999999</v>
+      </c>
+      <c r="H38">
+        <v>4788</v>
+      </c>
+      <c r="I38">
+        <v>27.872985</v>
+      </c>
+      <c r="J38">
+        <v>2461</v>
+      </c>
+      <c r="K38" s="3">
+        <f>F38/H38-1</f>
+        <v>-0.54051796157059318</v>
+      </c>
+      <c r="L38" s="1">
+        <f>J38/F38-1</f>
+        <v>0.11863636363636365</v>
+      </c>
+      <c r="M38" s="3">
+        <f>G38/I38-1</f>
+        <v>-0.61159032661912605</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39" t="s">
         <v>19</v>
       </c>
-      <c r="E26">
-        <v>14</v>
-      </c>
-      <c r="F26">
-        <v>2912</v>
-      </c>
-      <c r="G26">
-        <v>16003</v>
-      </c>
-      <c r="H26">
-        <v>24224</v>
-      </c>
-      <c r="I26">
-        <v>8226</v>
-      </c>
-      <c r="K26" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.33937417437252315</v>
-      </c>
-      <c r="L26" s="3">
-        <f t="shared" si="3"/>
-        <v>-0.48597138036618137</v>
-      </c>
-    </row>
-    <row r="27" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C27" t="s">
-        <v>43</v>
-      </c>
-      <c r="D27" t="s">
-        <v>36</v>
-      </c>
-      <c r="E27">
-        <v>6</v>
-      </c>
-      <c r="F27">
-        <v>164</v>
-      </c>
-      <c r="G27">
-        <v>217</v>
-      </c>
-      <c r="H27">
-        <v>471</v>
-      </c>
-      <c r="I27">
-        <v>191</v>
-      </c>
-      <c r="K27" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.53927813163481952</v>
-      </c>
-      <c r="L27" s="3">
-        <f t="shared" si="3"/>
-        <v>-0.11981566820276501</v>
-      </c>
-    </row>
-    <row r="28" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C28" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" t="s">
-        <v>22</v>
-      </c>
-      <c r="E28">
-        <v>16</v>
-      </c>
-      <c r="F28">
-        <v>2688</v>
-      </c>
-      <c r="G28">
-        <v>20671</v>
-      </c>
-      <c r="H28">
-        <v>28018</v>
-      </c>
-      <c r="I28">
-        <v>11811</v>
-      </c>
-      <c r="K28" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.26222428438860734</v>
-      </c>
-      <c r="L28" s="3">
-        <f t="shared" si="3"/>
-        <v>-0.42861980552464807</v>
-      </c>
-    </row>
-    <row r="29" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C29" t="s">
-        <v>45</v>
-      </c>
-      <c r="D29" t="s">
-        <v>22</v>
-      </c>
-      <c r="E29">
-        <v>16</v>
-      </c>
-      <c r="F29">
-        <v>2688</v>
-      </c>
-      <c r="G29">
-        <v>9151</v>
-      </c>
-      <c r="H29">
-        <v>29280</v>
-      </c>
-      <c r="I29">
-        <v>10692</v>
-      </c>
-      <c r="K29" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.6874658469945355</v>
-      </c>
-      <c r="L29" s="1">
-        <f t="shared" si="3"/>
-        <v>0.1683968965140421</v>
-      </c>
-    </row>
-    <row r="30" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C30" t="s">
-        <v>46</v>
-      </c>
-      <c r="D30" t="s">
-        <v>22</v>
-      </c>
-      <c r="E30">
-        <v>20</v>
-      </c>
-      <c r="F30">
-        <v>684</v>
-      </c>
-      <c r="G30">
-        <v>4795</v>
-      </c>
-      <c r="H30">
-        <v>6308</v>
-      </c>
-      <c r="I30">
-        <v>5817</v>
-      </c>
-      <c r="K30" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.23985415345592898</v>
-      </c>
-      <c r="L30" s="1">
-        <f t="shared" si="3"/>
-        <v>0.21313868613138687</v>
-      </c>
-    </row>
-    <row r="31" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D31" t="s">
-        <v>22</v>
-      </c>
-      <c r="E31">
-        <v>20</v>
-      </c>
-      <c r="F31">
-        <v>684</v>
-      </c>
-      <c r="G31">
-        <v>4883</v>
-      </c>
-      <c r="H31">
-        <v>5807</v>
-      </c>
-      <c r="I31">
-        <v>5136</v>
-      </c>
-      <c r="K31" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.15911830549337003</v>
-      </c>
-      <c r="L31" s="1">
-        <f t="shared" si="3"/>
-        <v>5.1812410403440534E-2</v>
-      </c>
-    </row>
-    <row r="32" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C32" t="s">
-        <v>48</v>
-      </c>
-      <c r="D32" t="s">
-        <v>22</v>
-      </c>
-      <c r="E32">
-        <v>22</v>
-      </c>
-      <c r="F32">
-        <v>3240</v>
-      </c>
-      <c r="G32">
-        <v>39569</v>
-      </c>
-      <c r="H32">
-        <v>35792</v>
-      </c>
-      <c r="I32">
-        <v>45769</v>
-      </c>
-      <c r="K32" s="1">
-        <f t="shared" si="2"/>
-        <v>0.10552637460885106</v>
-      </c>
-      <c r="L32" s="1">
-        <f t="shared" si="3"/>
-        <v>0.15668831661148874</v>
-      </c>
-    </row>
-    <row r="33" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C33" t="s">
-        <v>49</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="D39">
+        <v>12</v>
+      </c>
+      <c r="E39">
+        <v>640</v>
+      </c>
+      <c r="F39">
+        <v>2301</v>
+      </c>
+      <c r="G39">
+        <v>14.329871000000001</v>
+      </c>
+      <c r="H39">
+        <v>4884</v>
+      </c>
+      <c r="I39">
+        <v>32.869433999999998</v>
+      </c>
+      <c r="J39">
+        <v>2415</v>
+      </c>
+      <c r="K39" s="3">
+        <f>F39/H39-1</f>
+        <v>-0.52886977886977893</v>
+      </c>
+      <c r="L39" s="1">
+        <f>J39/F39-1</f>
+        <v>4.9543676662320735E-2</v>
+      </c>
+      <c r="M39" s="3">
+        <f>G39/I39-1</f>
+        <v>-0.56403657574389632</v>
+      </c>
+    </row>
+    <row r="40" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" t="s">
         <v>19</v>
       </c>
-      <c r="E33">
-        <v>12</v>
-      </c>
-      <c r="F33">
-        <v>640</v>
-      </c>
-      <c r="G33">
-        <v>2608</v>
-      </c>
-      <c r="H33">
-        <v>4250</v>
-      </c>
-      <c r="I33">
-        <v>3134</v>
-      </c>
-      <c r="K33" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.38635294117647057</v>
-      </c>
-      <c r="L33" s="1">
-        <f t="shared" si="3"/>
-        <v>0.20168711656441718</v>
-      </c>
-    </row>
-    <row r="34" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C34" t="s">
-        <v>50</v>
-      </c>
-      <c r="D34" t="s">
-        <v>22</v>
-      </c>
-      <c r="E34">
-        <v>22</v>
-      </c>
-      <c r="F34">
-        <v>3240</v>
-      </c>
-      <c r="G34">
-        <v>26858</v>
-      </c>
-      <c r="H34">
-        <v>33673</v>
-      </c>
-      <c r="I34">
-        <v>15811</v>
-      </c>
-      <c r="K34" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.20238766964630417</v>
-      </c>
-      <c r="L34" s="3">
-        <f t="shared" si="3"/>
-        <v>-0.41131134112741086</v>
-      </c>
-    </row>
-    <row r="35" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C35" t="s">
-        <v>51</v>
-      </c>
-      <c r="D35" t="s">
-        <v>19</v>
-      </c>
-      <c r="E35">
-        <v>12</v>
-      </c>
-      <c r="F35">
-        <v>640</v>
-      </c>
-      <c r="G35">
-        <v>2257</v>
-      </c>
-      <c r="H35">
-        <v>4331</v>
-      </c>
-      <c r="I35">
-        <v>2072</v>
-      </c>
-      <c r="K35" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.47887323943661975</v>
-      </c>
-      <c r="L35" s="3">
-        <f t="shared" si="3"/>
-        <v>-8.1967213114754078E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C36" t="s">
-        <v>52</v>
-      </c>
-      <c r="D36" t="s">
-        <v>19</v>
-      </c>
-      <c r="E36">
+      <c r="D40">
         <v>10</v>
       </c>
-      <c r="F36">
+      <c r="E40">
         <v>630</v>
       </c>
-      <c r="G36">
-        <v>1458</v>
-      </c>
-      <c r="H36">
+      <c r="F40">
+        <v>1432</v>
+      </c>
+      <c r="G40">
+        <v>6.5269760000000003</v>
+      </c>
+      <c r="H40">
         <v>3472</v>
       </c>
-      <c r="I36">
-        <v>1396</v>
-      </c>
-      <c r="K36" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.58006912442396308</v>
-      </c>
-      <c r="L36" s="3">
-        <f t="shared" si="3"/>
-        <v>-4.2524005486968441E-2</v>
-      </c>
-    </row>
-    <row r="37" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C37" t="s">
-        <v>53</v>
-      </c>
-      <c r="D37" t="s">
-        <v>22</v>
-      </c>
-      <c r="E37">
-        <v>18</v>
-      </c>
-      <c r="F37">
-        <v>2950</v>
-      </c>
-      <c r="G37">
-        <v>16842</v>
-      </c>
-      <c r="H37">
-        <v>35602</v>
-      </c>
-      <c r="I37">
-        <v>15307</v>
-      </c>
-      <c r="K37" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.52693668895005896</v>
-      </c>
-      <c r="L37" s="3">
-        <f t="shared" si="3"/>
-        <v>-9.1141194632466505E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C38" t="s">
-        <v>54</v>
-      </c>
-      <c r="D38" t="s">
-        <v>22</v>
-      </c>
-      <c r="E38">
-        <v>16</v>
-      </c>
-      <c r="F38">
-        <v>2340</v>
-      </c>
-      <c r="G38">
-        <v>19767</v>
-      </c>
-      <c r="H38">
-        <v>25280</v>
-      </c>
-      <c r="I38">
-        <v>11460</v>
-      </c>
-      <c r="K38" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.21807753164556964</v>
-      </c>
-      <c r="L38" s="3">
-        <f t="shared" si="3"/>
-        <v>-0.42024586431932009</v>
-      </c>
-    </row>
-    <row r="39" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C39" t="s">
-        <v>55</v>
-      </c>
-      <c r="D39" t="s">
-        <v>22</v>
-      </c>
-      <c r="E39">
-        <v>16</v>
-      </c>
-      <c r="F39">
-        <v>2340</v>
-      </c>
-      <c r="G39">
-        <v>8583</v>
-      </c>
-      <c r="H39">
-        <v>23182</v>
-      </c>
-      <c r="I39">
-        <v>9384</v>
-      </c>
-      <c r="K39" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.62975584505219562</v>
-      </c>
-      <c r="L39" s="1">
-        <f t="shared" si="3"/>
-        <v>9.3324012583013038E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C40" t="s">
-        <v>56</v>
-      </c>
-      <c r="D40" t="s">
-        <v>19</v>
-      </c>
-      <c r="E40">
-        <v>12</v>
-      </c>
-      <c r="F40">
-        <v>640</v>
-      </c>
-      <c r="G40">
-        <v>2207</v>
-      </c>
-      <c r="H40">
-        <v>4788</v>
-      </c>
       <c r="I40">
-        <v>2026</v>
+        <v>19.445034</v>
+      </c>
+      <c r="J40">
+        <v>1468</v>
       </c>
       <c r="K40" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.53905597326649957</v>
-      </c>
-      <c r="L40" s="3">
-        <f t="shared" si="3"/>
-        <v>-8.2011780697779812E-2</v>
-      </c>
-    </row>
-    <row r="41" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C41" t="s">
-        <v>57</v>
-      </c>
-      <c r="D41" t="s">
-        <v>19</v>
-      </c>
-      <c r="E41">
-        <v>12</v>
-      </c>
-      <c r="F41">
-        <v>640</v>
-      </c>
-      <c r="G41">
-        <v>2452</v>
-      </c>
-      <c r="H41">
-        <v>4884</v>
-      </c>
-      <c r="I41">
-        <v>2355</v>
-      </c>
-      <c r="K41" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.49795249795249796</v>
-      </c>
-      <c r="L41" s="3">
-        <f t="shared" si="3"/>
-        <v>-3.9559543230016314E-2</v>
-      </c>
-    </row>
-    <row r="42" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="C42" t="s">
-        <v>58</v>
-      </c>
-      <c r="D42" t="s">
-        <v>19</v>
-      </c>
-      <c r="E42">
-        <v>10</v>
-      </c>
-      <c r="F42">
-        <v>630</v>
-      </c>
-      <c r="G42">
-        <v>1458</v>
-      </c>
-      <c r="H42">
-        <v>3472</v>
-      </c>
-      <c r="I42">
-        <v>1396</v>
-      </c>
-      <c r="K42" s="3">
-        <f t="shared" si="2"/>
-        <v>-0.58006912442396308</v>
-      </c>
-      <c r="L42" s="3">
-        <f t="shared" si="3"/>
-        <v>-4.2524005486968441E-2</v>
-      </c>
-    </row>
-    <row r="43" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="K43" s="1"/>
+        <f>F40/H40-1</f>
+        <v>-0.5875576036866359</v>
+      </c>
+      <c r="L40" s="1">
+        <f>J40/F40-1</f>
+        <v>2.5139664804469275E-2</v>
+      </c>
+      <c r="M40" s="3">
+        <f>G40/I40-1</f>
+        <v>-0.66433712586977212</v>
+      </c>
+    </row>
+    <row r="41" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="K41" s="3"/>
+      <c r="L41" s="1"/>
+      <c r="M41" s="3"/>
+    </row>
+    <row r="42" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="K42" s="3"/>
+      <c r="L42" s="1"/>
+      <c r="M42" s="3"/>
+    </row>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="K43" s="3"/>
       <c r="L43" s="1"/>
-    </row>
-    <row r="44" spans="3:12" x14ac:dyDescent="0.2">
-      <c r="K44" s="1"/>
+      <c r="M43" s="3"/>
+    </row>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="K44" s="3"/>
       <c r="L44" s="1"/>
+      <c r="M44" s="3"/>
+    </row>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="K45" s="3"/>
+      <c r="L45" s="1"/>
+      <c r="M45" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>